<commit_message>
fix: resolve auto-dispatch credit matching and layout hydration issues
- Rewrote generateBookings to fix credit ID mapping and syntax errors
- Updated import logic to default records to 'Approved' status
- Increased axios timeouts to 10 minutes for batch operations
- Removed redundant status badges from service requests table
- Fixed hydration warnings and set language to English
</commit_message>
<xml_diff>
--- a/test-service-requests.xlsx
+++ b/test-service-requests.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="5CN_Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Service Requests" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -64,9 +64,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -398,365 +397,438 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S6"/>
+  <dimension ref="A1:V6"/>
+  <cols>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="15.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="50.83203125" customWidth="1"/>
+    <col min="5" max="5" width="15.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="30.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="12.83203125" customWidth="1"/>
+    <col min="11" max="11" width="15.83203125" customWidth="1"/>
+    <col min="12" max="12" width="12.83203125" customWidth="1"/>
+    <col min="13" max="13" width="15.83203125" customWidth="1"/>
+    <col min="14" max="14" width="20.83203125" customWidth="1"/>
+    <col min="15" max="15" width="25.83203125" customWidth="1"/>
+    <col min="16" max="16" width="12.83203125" customWidth="1"/>
+    <col min="17" max="17" width="12.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Mr_no</v>
+        <v>Name</v>
       </c>
       <c r="B1" t="str">
-        <v xml:space="preserve">ID number </v>
+        <v>MobileNumber</v>
       </c>
       <c r="C1" t="str">
-        <v>Patient_Name</v>
+        <v>Mobile_Number</v>
       </c>
       <c r="D1" t="str">
+        <v>Country Code</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Address</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Location</v>
+      </c>
+      <c r="G1" t="str">
+        <v>ApprovedService</v>
+      </c>
+      <c r="H1" t="str">
         <v>Approved Service</v>
       </c>
-      <c r="E1" t="str">
+      <c r="I1" t="str">
+        <v>Service</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Recurring Period</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Expiry Date</v>
+      </c>
+      <c r="L1" t="str">
+        <v>ApprovedCount</v>
+      </c>
+      <c r="M1" t="str">
         <v>Approved_Count</v>
       </c>
-      <c r="F1" t="str">
+      <c r="N1" t="str">
         <v>Used_Count</v>
       </c>
-      <c r="G1" t="str">
+      <c r="O1" t="str">
         <v>Remaining_Count</v>
       </c>
-      <c r="H1" t="str">
-        <v>Approval_Start_Date</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Approval_Expiry_Date</v>
-      </c>
-      <c r="J1" t="str">
-        <v>Address</v>
-      </c>
-      <c r="K1" t="str">
-        <v>Location</v>
-      </c>
-      <c r="L1" t="str">
-        <v>Latitude</v>
-      </c>
-      <c r="M1" t="str">
-        <v>Longitude</v>
-      </c>
-      <c r="N1" t="str">
-        <v>Country_Code</v>
-      </c>
-      <c r="O1" t="str">
-        <v>Mobile_Number</v>
-      </c>
       <c r="P1" t="str">
-        <v>File_Number</v>
+        <v>Notes</v>
       </c>
       <c r="Q1" t="str">
-        <v>Insurance_Number</v>
+        <v>Start Time</v>
       </c>
       <c r="R1" t="str">
-        <v>Level_of_Care</v>
+        <v>End Time</v>
       </c>
       <c r="S1" t="str">
-        <v>Recurring period (Days)</v>
+        <v>Preferred Staff</v>
+      </c>
+      <c r="T1" t="str">
+        <v>Preferred Days</v>
+      </c>
+      <c r="U1" t="str">
+        <v>Lat</v>
+      </c>
+      <c r="V1" t="str">
+        <v>Lng</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>99923501</v>
+        <v>Test Customer 1</v>
       </c>
       <c r="B2" t="str">
-        <v>9995465001</v>
+        <v>99990101</v>
       </c>
       <c r="C2" t="str">
-        <v>Test Customer 1</v>
+        <v>99990101</v>
       </c>
       <c r="D2" t="str">
+        <v>SA</v>
+      </c>
+      <c r="E2" t="str">
+        <v>King Fahd Road, Al Olaya, Riyadh 12211, Saudi Arabia</v>
+      </c>
+      <c r="F2" t="str">
+        <v>King Fahd Road, Al Olaya, Riyadh 12211, Saudi Arabia</v>
+      </c>
+      <c r="G2" t="str">
         <v>GP</v>
       </c>
-      <c r="E2">
+      <c r="H2" t="str">
+        <v>GP</v>
+      </c>
+      <c r="I2" t="str">
+        <v>GP</v>
+      </c>
+      <c r="J2" t="str">
+        <v>30 days</v>
+      </c>
+      <c r="K2" t="str">
+        <v>2026-02-14</v>
+      </c>
+      <c r="L2">
         <v>10</v>
       </c>
-      <c r="F2">
-        <v>9</v>
-      </c>
-      <c r="G2">
-        <v>1</v>
-      </c>
-      <c r="H2" s="1">
-        <v>46035</v>
-      </c>
-      <c r="I2" s="1">
-        <v>46042</v>
-      </c>
-      <c r="J2" t="str">
-        <v>2716 Olaya St, Al Wurud, Riyadh 12251, Saudi Arabia</v>
-      </c>
-      <c r="K2" t="str">
-        <v>24.7136,46.6753</v>
-      </c>
-      <c r="L2">
+      <c r="M2">
+        <v>10</v>
+      </c>
+      <c r="N2">
+        <v>0</v>
+      </c>
+      <c r="O2">
+        <v>10</v>
+      </c>
+      <c r="P2" t="str">
+        <v>Regular checkup appointment</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>09:00</v>
+      </c>
+      <c r="R2" t="str">
+        <v>17:00</v>
+      </c>
+      <c r="S2" t="str">
+        <v/>
+      </c>
+      <c r="T2" t="str">
+        <v>Monday,Wednesday,Friday</v>
+      </c>
+      <c r="U2">
         <v>24.7136</v>
       </c>
-      <c r="M2">
+      <c r="V2">
         <v>46.6753</v>
-      </c>
-      <c r="N2">
-        <v>966</v>
-      </c>
-      <c r="O2">
-        <v>99990101</v>
-      </c>
-      <c r="P2">
-        <v>99960</v>
-      </c>
-      <c r="Q2" t="str">
-        <v>99923501</v>
-      </c>
-      <c r="R2" t="str">
-        <v>PACT1</v>
-      </c>
-      <c r="S2">
-        <v>2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>99923502</v>
+        <v>Test Customer 2</v>
       </c>
       <c r="B3" t="str">
-        <v>9995465002</v>
+        <v>99990102</v>
       </c>
       <c r="C3" t="str">
-        <v>Test Customer 2</v>
+        <v>99990102</v>
       </c>
       <c r="D3" t="str">
+        <v>SA</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Al Malaz, Riyadh 12613, Saudi Arabia</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Al Malaz, Riyadh 12613, Saudi Arabia</v>
+      </c>
+      <c r="G3" t="str">
         <v>Nursing</v>
       </c>
-      <c r="E3">
-        <v>10</v>
-      </c>
-      <c r="F3">
-        <v>9</v>
-      </c>
-      <c r="G3">
-        <v>1</v>
-      </c>
-      <c r="H3" s="1">
-        <v>46035</v>
-      </c>
-      <c r="I3" s="1">
-        <v>46042</v>
+      <c r="H3" t="str">
+        <v>Nursing</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Nursing</v>
       </c>
       <c r="J3" t="str">
-        <v>RMDD8074، 8074 جبل نهير، 2185, Ad Dar Al Baida, Riyadh 14518, Saudi Arabia</v>
+        <v>14 days</v>
       </c>
       <c r="K3" t="str">
-        <v>24.6877,46.7215</v>
+        <v>2026-02-14</v>
       </c>
       <c r="L3">
-        <v>24.6877</v>
+        <v>20</v>
       </c>
       <c r="M3">
-        <v>46.7215</v>
+        <v>20</v>
       </c>
       <c r="N3">
-        <v>966</v>
+        <v>5</v>
       </c>
       <c r="O3">
-        <v>99990102</v>
-      </c>
-      <c r="P3">
-        <v>99961</v>
+        <v>15</v>
+      </c>
+      <c r="P3" t="str">
+        <v>Home care service</v>
       </c>
       <c r="Q3" t="str">
-        <v>99923502</v>
+        <v>08:00</v>
       </c>
       <c r="R3" t="str">
-        <v>LTCA</v>
-      </c>
-      <c r="S3">
-        <v>2</v>
+        <v>16:00</v>
+      </c>
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3" t="str">
+        <v>Tuesday,Thursday</v>
+      </c>
+      <c r="U3">
+        <v>24.6408</v>
+      </c>
+      <c r="V3">
+        <v>46.7214</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>99923503</v>
+        <v>Test Customer 3</v>
       </c>
       <c r="B4" t="str">
-        <v>9995465003</v>
+        <v>99990103</v>
       </c>
       <c r="C4" t="str">
-        <v>Test Customer 3</v>
+        <v>99990103</v>
       </c>
       <c r="D4" t="str">
+        <v>SA</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Al Murabba, Riyadh 12613, Saudi Arabia</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Al Murabba, Riyadh 12613, Saudi Arabia</v>
+      </c>
+      <c r="G4" t="str">
         <v>GP</v>
       </c>
-      <c r="E4">
-        <v>10</v>
-      </c>
-      <c r="F4">
-        <v>9</v>
-      </c>
-      <c r="G4">
-        <v>1</v>
-      </c>
-      <c r="H4" s="1">
-        <v>46035</v>
-      </c>
-      <c r="I4" s="1">
-        <v>46042</v>
+      <c r="H4" t="str">
+        <v>GP</v>
+      </c>
+      <c r="I4" t="str">
+        <v>GP</v>
       </c>
       <c r="J4" t="str">
-        <v>RQJA2976, 2976 No.4, 8167، حي الجزيرة، Riyadh 14261, Saudi Arabia</v>
+        <v>1 month</v>
       </c>
       <c r="K4" t="str">
-        <v>24.7574,46.6428</v>
+        <v>2026-02-14</v>
       </c>
       <c r="L4">
-        <v>24.7574</v>
+        <v>5</v>
       </c>
       <c r="M4">
-        <v>46.6428</v>
+        <v>5</v>
       </c>
       <c r="N4">
-        <v>966</v>
+        <v>2</v>
       </c>
       <c r="O4">
-        <v>99990103</v>
-      </c>
-      <c r="P4">
-        <v>99962</v>
+        <v>3</v>
+      </c>
+      <c r="P4" t="str">
+        <v>Monthly consultation</v>
       </c>
       <c r="Q4" t="str">
-        <v>99923503</v>
+        <v>10:00</v>
       </c>
       <c r="R4" t="str">
-        <v>PACT1</v>
-      </c>
-      <c r="S4">
-        <v>2</v>
+        <v>18:00</v>
+      </c>
+      <c r="S4" t="str">
+        <v/>
+      </c>
+      <c r="T4" t="str">
+        <v>Monday,Wednesday</v>
+      </c>
+      <c r="U4">
+        <v>24.65</v>
+      </c>
+      <c r="V4">
+        <v>46.71</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>99923504</v>
+        <v>Test Customer 4</v>
       </c>
       <c r="B5" t="str">
-        <v>9995465004</v>
+        <v>99990104</v>
       </c>
       <c r="C5" t="str">
-        <v>Test Customer 4</v>
+        <v>99990104</v>
       </c>
       <c r="D5" t="str">
+        <v>SA</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Al Wurud, Riyadh 12251, Saudi Arabia</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Al Wurud, Riyadh 12251, Saudi Arabia</v>
+      </c>
+      <c r="G5" t="str">
         <v>RT</v>
       </c>
-      <c r="E5">
-        <v>10</v>
-      </c>
-      <c r="F5">
-        <v>9</v>
-      </c>
-      <c r="G5">
-        <v>1</v>
-      </c>
-      <c r="H5" s="1">
-        <v>46035</v>
-      </c>
-      <c r="I5" s="1">
-        <v>46042</v>
+      <c r="H5" t="str">
+        <v>RT</v>
+      </c>
+      <c r="I5" t="str">
+        <v>RT</v>
       </c>
       <c r="J5" t="str">
-        <v>RSNB3234, 3234 At Tanukhi, 7111, Ar Rimayah, Riyadh 14816, Saudi Arabia</v>
+        <v>7 days</v>
       </c>
       <c r="K5" t="str">
-        <v>24.6833,46.6167</v>
+        <v>2026-02-14</v>
       </c>
       <c r="L5">
-        <v>24.6833</v>
+        <v>15</v>
       </c>
       <c r="M5">
-        <v>46.6167</v>
+        <v>15</v>
       </c>
       <c r="N5">
-        <v>966</v>
+        <v>0</v>
       </c>
       <c r="O5">
-        <v>99990104</v>
-      </c>
-      <c r="P5">
-        <v>99963</v>
+        <v>15</v>
+      </c>
+      <c r="P5" t="str">
+        <v/>
       </c>
       <c r="Q5" t="str">
-        <v>99923504</v>
+        <v>09:00</v>
       </c>
       <c r="R5" t="str">
-        <v>LTCA</v>
-      </c>
-      <c r="S5">
-        <v>2</v>
+        <v>17:00</v>
+      </c>
+      <c r="S5" t="str">
+        <v/>
+      </c>
+      <c r="T5" t="str">
+        <v/>
+      </c>
+      <c r="U5">
+        <v>24.7136</v>
+      </c>
+      <c r="V5">
+        <v>46.6753</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>99923505</v>
+        <v>Test Customer 5</v>
       </c>
       <c r="B6" t="str">
-        <v>9995465005</v>
+        <v>99990105</v>
       </c>
       <c r="C6" t="str">
-        <v>Test Customer 5</v>
+        <v>99990105</v>
       </c>
       <c r="D6" t="str">
+        <v>SA</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Al Nakheel, Riyadh 12382, Saudi Arabia</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Al Nakheel, Riyadh 12382, Saudi Arabia</v>
+      </c>
+      <c r="G6" t="str">
         <v>Nursing</v>
       </c>
-      <c r="E6">
-        <v>10</v>
-      </c>
-      <c r="F6">
+      <c r="H6" t="str">
+        <v>Nursing</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Nursing</v>
+      </c>
+      <c r="J6" t="str">
+        <v>21 days</v>
+      </c>
+      <c r="K6" t="str">
+        <v>2026-02-14</v>
+      </c>
+      <c r="L6">
+        <v>12</v>
+      </c>
+      <c r="M6">
+        <v>12</v>
+      </c>
+      <c r="N6">
+        <v>3</v>
+      </c>
+      <c r="O6">
         <v>9</v>
       </c>
-      <c r="G6">
-        <v>1</v>
-      </c>
-      <c r="H6" s="1">
-        <v>46035</v>
-      </c>
-      <c r="I6" s="1">
-        <v>46042</v>
-      </c>
-      <c r="J6" t="str">
-        <v>PM7G+C4F, Al Olaya, Riyadh 12251, Saudi Arabia</v>
-      </c>
-      <c r="K6" t="str">
-        <v>24.6982,46.6856</v>
-      </c>
-      <c r="L6">
+      <c r="P6" t="str">
+        <v>Follow-up appointment</v>
+      </c>
+      <c r="Q6" t="str">
+        <v>08:30</v>
+      </c>
+      <c r="R6" t="str">
+        <v>16:30</v>
+      </c>
+      <c r="S6" t="str">
+        <v/>
+      </c>
+      <c r="T6" t="str">
+        <v>Monday,Wednesday,Friday</v>
+      </c>
+      <c r="U6">
         <v>24.6982</v>
       </c>
-      <c r="M6">
+      <c r="V6">
         <v>46.6856</v>
-      </c>
-      <c r="N6">
-        <v>966</v>
-      </c>
-      <c r="O6">
-        <v>99990105</v>
-      </c>
-      <c r="P6">
-        <v>99964</v>
-      </c>
-      <c r="Q6" t="str">
-        <v>99923505</v>
-      </c>
-      <c r="R6" t="str">
-        <v>PACT1</v>
-      </c>
-      <c r="S6">
-        <v>2</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>